<commit_message>
fix: clean fictional test packet entities
</commit_message>
<xml_diff>
--- a/test_sets/deals/packet_5_vanguard_aerospace_renegotiate/Vanguard_Aerospace_Customer_Concentration_AR.xlsx
+++ b/test_sets/deals/packet_5_vanguard_aerospace_renegotiate/Vanguard_Aerospace_Customer_Concentration_AR.xlsx
@@ -587,12 +587,12 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Lockheed Martin Aeronautics</t>
+          <t>Fabrikam Aerostructures</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>F-35 Structural Brackets</t>
+          <t>AX-114 Structural Brackets</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
@@ -615,7 +615,7 @@
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Raytheon Missile Systems</t>
+          <t>Adatum Guidance Systems</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -643,7 +643,7 @@
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>General Dynamics Land Systems</t>
+          <t>Contoso Land Systems</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -671,7 +671,7 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Northrop Grumman Tooling</t>
+          <t>Proseware Precision Tooling</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -699,7 +699,7 @@
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Boeing Defense Subcontractor</t>
+          <t>Tailspin Defense Group</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">

</xml_diff>